<commit_message>
Spreadsheets: keep Excel column widths, hide hidden rows/columns, CSV fixes; test-pack file fixes
- Columns keep their Excel widths (table width is now fixed); text runs on into
  empty cells to its right like Excel; full text on hover when cut off
- Hidden rows and columns are no longer shown
- CSV: columns sized to their content (max 420 px), line breaks inside a cell shown
- Online counter: page-type update also sends the timestamp (no permission warning)
- Test pack: Word page 7 back to one column (one <w:cols> per section), PDF gradient
  clipped to its box, 16-bit TIFF uses the full gray range, Excel column B wider
</commit_message>
<xml_diff>
--- a/public/samples/test-pack/test-excel.xlsx
+++ b/public/samples/test-pack/test-excel.xlsx
@@ -1747,7 +1747,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2024,7 +2025,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2326,7 +2328,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="6" width="9" hidden="1" customWidth="1"/>
   </cols>
@@ -2615,7 +2618,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2784,7 +2788,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2917,7 +2922,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5792CE74-CC52-493A-A4E7-351B641232EE}</x14:id>
+          <x14:id>{0D4EC1DA-03B8-4F75-A6C3-DD0B3B37B885}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -2943,7 +2948,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5792CE74-CC52-493A-A4E7-351B641232EE}">
+          <x14:cfRule type="dataBar" id="{0D4EC1DA-03B8-4F75-A6C3-DD0B3B37B885}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -2963,7 +2968,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Test checklist results; spreadsheet fixes; test-pack file fixes
- TEST-CHECKLIST.xlsx: all 506 tests run on Stage and Angular; Result, notes and
  test date filled in; Summary shows Pass / Fail per file
- Columns keep their Excel widths (table width is now fixed); text runs on into
  empty cells to its right like Excel; full text on hover when cut off
- Hidden rows and columns are no longer shown
- CSV: columns sized to their content (max 420 px), line breaks inside a cell shown
- Online counter: page-type update also sends the timestamp (no permission warning)
- Test pack: Word page 7 back to one column (one <w:cols> per section), PDF gradient
  clipped to its box, 16-bit TIFF uses the full gray range, Excel column B wider
</commit_message>
<xml_diff>
--- a/public/samples/test-pack/test-excel.xlsx
+++ b/public/samples/test-pack/test-excel.xlsx
@@ -1747,7 +1747,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2024,7 +2025,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2326,7 +2328,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
     <col min="6" max="6" width="9" hidden="1" customWidth="1"/>
   </cols>
@@ -2615,7 +2618,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2784,7 +2788,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2917,7 +2922,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5792CE74-CC52-493A-A4E7-351B641232EE}</x14:id>
+          <x14:id>{0D4EC1DA-03B8-4F75-A6C3-DD0B3B37B885}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -2943,7 +2948,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5792CE74-CC52-493A-A4E7-351B641232EE}">
+          <x14:cfRule type="dataBar" id="{0D4EC1DA-03B8-4F75-A6C3-DD0B3B37B885}">
             <x14:dataBar minLength="0" maxLength="100">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>
@@ -2963,7 +2968,8 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>